<commit_message>
Adaugare task-uri realizate cu ajutorul Stream API
</commit_message>
<xml_diff>
--- a/fisier.xlsx
+++ b/fisier.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
   <si>
     <t>3574</t>
   </si>
@@ -41,6 +41,12 @@
     <t>Ioana</t>
   </si>
   <si>
+    <t>3531</t>
+  </si>
+  <si>
+    <t>Matei</t>
+  </si>
+  <si>
     <t>3573</t>
   </si>
   <si>
@@ -66,9 +72,6 @@
   </si>
   <si>
     <t>Ionescu</t>
-  </si>
-  <si>
-    <t>Matei</t>
   </si>
   <si>
     <t>C221</t>
@@ -131,7 +134,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -184,66 +187,80 @@
         <v>10</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="D5" t="s" s="0">
         <v>14</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="C6" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="C6" t="s" s="0">
-        <v>18</v>
-      </c>
       <c r="D6" t="s" s="0">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D7" t="s" s="0">
         <v>20</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="D8" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="C8" t="s" s="0">
+      <c r="B9" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="D8" t="s" s="0">
-        <v>19</v>
+      <c r="D9" t="s" s="0">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>